<commit_message>
Implement multiple page object framework and Cucumber E2E flow
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/TestData.xlsx
+++ b/src/test/resources/testData/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Balaji\Desktop\AutomationProject\myAutomationProject\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C260C73-AF30-48CC-A2B9-A5E124C9BC44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8976C8B-29B6-42F7-90E9-DD4958E68DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
   <si>
     <t>standard_user</t>
   </si>
@@ -82,6 +82,42 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Sauce Labs Backpack</t>
+  </si>
+  <si>
+    <t>Sauce Labs Fleece Jacket</t>
+  </si>
+  <si>
+    <t>Sauce Labs Onesie</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>ZipCode</t>
+  </si>
+  <si>
+    <t>Balaji</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>Ganesamurthy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balaji </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ganesamurthy </t>
   </si>
 </sst>
 </file>
@@ -150,11 +186,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -435,111 +480,183 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="25.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="8.88671875" style="3"/>
+    <col min="2" max="2" width="25.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="4">
+        <v>600001</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>17</v>
+      <c r="D4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="4">
+        <v>600001</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="4">
+        <v>600001</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="4">
+        <v>600001</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>